<commit_message>
Added all the backend Files
</commit_message>
<xml_diff>
--- a/backend/Data/finaldata.xlsx
+++ b/backend/Data/finaldata.xlsx
@@ -448,12 +448,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Black Sea Corn Financially Settled (Platts) Options</t>
+          <t>BTIC on S&amp;P-GSCI Commodity Index Futures</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BSO</t>
+          <t>GDT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -465,12 +465,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Chicago SRW Wheat TAS Futures</t>
+          <t>Cash-Settled Cheese Futures</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ZWT</t>
+          <t>CSC</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -482,12 +482,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Options on Lumber Futures</t>
+          <t>Chicago SRW Wheat-Corn ICS Synthetic Futures</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LBR</t>
+          <t>QCW</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -499,12 +499,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Corn Mar-Jul CSO</t>
+          <t>Urea US Gulf Options</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CZ7</t>
+          <t>UGO</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -516,12 +516,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Soybean Meal Sep-Dec CSO</t>
+          <t>DAP FOB NOLA Futures</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MC5</t>
+          <t>DFN</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -533,12 +533,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BTIC on S&amp;P-GSCI Excess Return Index Futures</t>
+          <t>Soybean Nov-July CSO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>GIT</t>
+          <t>SZ9</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -550,12 +550,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Class IV Milk Options</t>
+          <t>Oats Options</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GDK</t>
+          <t>OZO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -567,12 +567,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cash-Settled Cheese Futures</t>
+          <t>MGEX-Chicago SRW Wheat Spread Synthetic Futures</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CSC</t>
+          <t>MCX</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -584,12 +584,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Consecutive KC HRW CSO</t>
+          <t>Soybean Oil Futures</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KZC</t>
+          <t>ZL</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -601,12 +601,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Soybean Meal Aug-Dec CSO</t>
+          <t>Consecutive Chicago SRW Wheat CSO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MC4</t>
+          <t>CZW</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -618,12 +618,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Soybean TAS Futures</t>
+          <t>Short-Dated New Crop Soybean Meal Options</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SBT</t>
+          <t>OMD</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -635,12 +635,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BTIC on Bitcoin Friday Futures</t>
+          <t>Monthly Options on Micro Ether Futures</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BFB</t>
+          <t>VM</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -652,12 +652,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BTIC on Ether Futures London Close</t>
+          <t>BTIC on Bitcoin Friday Futures</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ETB</t>
+          <t>BFB</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -669,12 +669,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BTIC on Ether Futures New York Close</t>
+          <t>BTIC on Bitcoin futures against APAC Close (Bitcoin Reference Rate APAC - BRRAP)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ENB</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -686,12 +686,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Micro Ether Futures</t>
+          <t>TAS on Bitcoin Futures</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>TBT</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -703,12 +703,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Micro Bitcoin Futures</t>
+          <t>Monthly Options on Micro Bitcoin Futures</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MBT</t>
+          <t>WM</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -720,12 +720,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BTIC on Micro Ether Futures New York Close</t>
+          <t>BTIC on Micro Bitcoin Futures New York Close</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>EYB</t>
+          <t>MYB</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -737,12 +737,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Options on Ether Futures</t>
+          <t>Bitcoin Friday Futures</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>BFF</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -754,12 +754,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Bitcoin Friday Futures</t>
+          <t>BTIC on Micro Ether Futures New York Close</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BFF</t>
+          <t>EYB</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -771,12 +771,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ether Futures</t>
+          <t>Micro Bitcoin Euro Futures</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>EBM</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -788,12 +788,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BTIC on Bitcoin futures against APAC Close (Bitcoin Reference Rate APAC - BRRAP)</t>
+          <t>BTIC on Micro Ether Futures London Close</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>EMB</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -805,12 +805,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BTIC on Micro Bitcoin Futures London Close</t>
+          <t>Micro Ether Euro Futures</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MIB</t>
+          <t>EEM</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -822,12 +822,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Micro WTI Crude Oil Futures</t>
+          <t>Bakken Cushing (Argus) vs. WTI Trade Month Futures</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MCL</t>
+          <t>BKT</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -839,12 +839,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PJM West Hub 50 MW Same Day Option D04</t>
+          <t>Gasoil 0.1% Cargoes CIF NWE (Platts) vs. Low Sulphur Gasoil BALMO Futures</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Z04</t>
+          <t>4V</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -856,12 +856,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Freight Route Middle East to China (TD3C) (Baltic) Average Price Option</t>
+          <t>Mini Japan C&amp;F Naphtha (Platts) Futures</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>TDT</t>
+          <t>MJN</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -873,12 +873,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Dated Brent (Platts) Daily Futures</t>
+          <t>PJM METED Zone Off-Peak Calendar-Month Day-Ahead LMP Futures</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>A7G</t>
+          <t>A46</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -907,12 +907,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Natural Gas Short-Term Option D11</t>
+          <t>NY Harbor ULSD BALMO Futures</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>U11</t>
+          <t>A1G</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -924,12 +924,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Natural Gas Short-Term Option D09</t>
+          <t>Los Angeles CARB Diesel (OPIS) Futures</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>U09</t>
+          <t>ALX</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -941,12 +941,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ISO New England Rhode Island Zone Peak Calendar-Day 5 MW Day-Ahead LMP Futures</t>
+          <t>Mini Gasoil 0.1% Cargoes CIF NWE (Platts) vs. Low Sulphur Gasoil Futures</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>NRP</t>
+          <t>MGF</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -958,12 +958,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>European FOB Rdam Marine Fuel 0.5% Barges (Platts) Futures</t>
+          <t>Micro Crude Oil TAS</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>R5F</t>
+          <t>MCT</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -975,12 +975,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Gulf Coast CBOB Gasoline A2 (Platts) Futures</t>
+          <t>ERCOT North 345 kV Hub 5 MW Peak Futures</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CRG</t>
+          <t>AI5</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -992,12 +992,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>HDPE High Density Polyethylene (PCW) BALMO Futures</t>
+          <t>Singapore Gasoline 92 Unleaded (Platts) vs Gasoline Eurobob Non-Oxy NWE Barges (Argus) Futures</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>HPD</t>
+          <t>SGF</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1009,12 +1009,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BTIC on Adjusted Interest Rate S&amp;P 500 Total Return (SOFR) Futures</t>
+          <t>BTIC FTSE 100 Index (GBP) Futures</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ASPT</t>
+          <t>FTT</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1026,12 +1026,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TMAC on E-mini Dow Jones Industrial Average Futures</t>
+          <t>E-mini FTSE Emerging Index Futures</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>YMX</t>
+          <t>EI</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1043,12 +1043,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>BTIC E-mini Nasdaq-100 Futures</t>
+          <t>BTIC on E-mini S&amp;P Oil &amp; Gas Exploration &amp; Production Select Industry Futures</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>NQT</t>
+          <t>SWT</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1060,12 +1060,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TACO+ Futures on E-mini S&amp;P 500 Stock Price Index Futures</t>
+          <t>E-mini Industrial Select Sector Futures</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EQ1</t>
+          <t>XAI</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1077,12 +1077,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>E-mini  Russell 2000 Value Index Futures</t>
+          <t>E-mini S&amp;P 500 Equal Weight Futures</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>R2V</t>
+          <t>EWF</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1094,12 +1094,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>BTIC on E-mini IPOX 100 U.S. Index Futures</t>
+          <t>BTIC on S&amp;P 500 Total Return Index Futures</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>IPT</t>
+          <t>TRB</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1111,12 +1111,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>BTIC E-mini FTSE China 50 Index Futures</t>
+          <t>S&amp;P 500 Growth Futures</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>FTC</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1128,12 +1128,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>E-mini FTSE Emerging Index Futures</t>
+          <t>Dow Jones Real Estate BTIC Futures</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EI</t>
+          <t>REX</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1145,12 +1145,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BTIC on Nikkei (USD) Futures</t>
+          <t>BTIC on E-mini Consumer Staples Select Sector Futures</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>NKT</t>
+          <t>XPT</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1162,12 +1162,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>E-mini  Russell 2000 Growth Index Futures</t>
+          <t>BTIC E-mini S&amp;P 500 Futures</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>R2G</t>
+          <t>EST</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1179,12 +1179,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>E-mini S&amp;P Insurance Select Industry Futures</t>
+          <t>E-mini Russell 2000 Index Futures</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SXI</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1196,12 +1196,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Euro/Australian Dollar Futures</t>
+          <t>Australian Dollar Futures</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>EAD</t>
+          <t>6A</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1213,12 +1213,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Micro GBP/USD Futures</t>
+          <t>Russian Ruble Futures</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>M6B</t>
+          <t>6R</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1230,12 +1230,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Indian Rupee/USD Futures</t>
+          <t>Czech Koruna/Euro (CZK/EUR) Cross Rate Futures</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SIR</t>
+          <t>ECK</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1247,12 +1247,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Euro/Canadian Dollar Futures</t>
+          <t>Chinese Renminbi/Euro Futures</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ECD</t>
+          <t>RME</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1264,12 +1264,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Japanese Yen Futures</t>
+          <t>Turkish Lira/US Dollar (TRY/USD) Future</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>6J</t>
+          <t>TRL</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1281,12 +1281,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>GBP/AUD Futures</t>
+          <t>USD/CNH Monthly Options</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PAD</t>
+          <t>CNH</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1298,12 +1298,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Euro/Swiss Franc Futures</t>
+          <t>Australian Dollar/Japanese Yen Futures</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>RF</t>
+          <t>AJY</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1315,12 +1315,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>EUR/JPY Monthly Options</t>
+          <t>Micro AUD/USD Futures</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>RY</t>
+          <t>M6A</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1332,12 +1332,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MXN/USD Monthly Options</t>
+          <t>New Zealand Dollar Futures</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>6M</t>
+          <t>6N</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1349,12 +1349,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Australian Dollar Futures</t>
+          <t>Brazilian Real Futures</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>6A</t>
+          <t>6L</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1366,12 +1366,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Swiss Franc/Japanese Yen Futures</t>
+          <t>Euro/Japanese Yen Futures</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SJY</t>
+          <t>RY</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1383,12 +1383,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BTIC on Bloomberg IG Credit Futures</t>
+          <t>5-Year MAC SOFR Swap Futures</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>IQBT</t>
+          <t>F1S</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1400,12 +1400,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>30-Year UMBS TBA Futures - 2.5% Coupon</t>
+          <t>5-Year Yield Futures</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>25U</t>
+          <t>5YY</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1417,12 +1417,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>30 Day Federal Funds 6 Month Midcurve Options</t>
+          <t>20-Year MAC SOFR Swap Futures</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ZQ6</t>
+          <t>E1S</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1434,12 +1434,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Euro Short-Term Rate (€STR) - Three-Month Single Contract Basis Spread Futures</t>
+          <t>30-Year UMBS TBA Futures - 4.5% Coupon</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EUS</t>
+          <t>45U</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1451,12 +1451,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>10-Year Yield Futures</t>
+          <t>2-Year Yield Futures</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>10Y</t>
+          <t>2YY</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1468,12 +1468,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>TAS on 2-Year Treasury Note Futures</t>
+          <t>30-Year UMBS TBA Futures - 2.0% Coupon</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ZTT</t>
+          <t>20U</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1485,12 +1485,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Three-Year Mid-Curve Options on Three-Month SOFR Futures</t>
+          <t>2-Year T-Note Options</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>OZT</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1502,12 +1502,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>TAS on 10-Year Treasury Note Futures</t>
+          <t>Ultra U.S. Treasury Bond Futures</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ZNS</t>
+          <t>UB</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1519,12 +1519,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>1-Year Eris SOFR Swap Futures</t>
+          <t>ESTR Futures</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>YIA</t>
+          <t>ESR</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1536,12 +1536,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>5-Year Yield Futures</t>
+          <t>2-Year MAC SOFR Swap Futures</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>5YY</t>
+          <t>T1S</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1553,12 +1553,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2-Year T-Note Futures</t>
+          <t>TAS on 2-Year Treasury Note Futures</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ZT</t>
+          <t>ZTT</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1570,12 +1570,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Copper Premium Grade A CIF Shanghai (Metal Bulletin) Futures</t>
+          <t>Micro Gold TAS Futures</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>CUP</t>
+          <t>MGT</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1587,12 +1587,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Micro Copper Futures</t>
+          <t>Shanghai Gold (USD) Futures</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MHG</t>
+          <t>SGU</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1604,12 +1604,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>E-mini Silver Futures</t>
+          <t>Spodumene CIF China (Fastmarkets) Futures</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>QI</t>
+          <t>SPM</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1621,12 +1621,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Aluminum A380 Alloy (Platts) Futures</t>
+          <t>Iron Ore 62% Fe, CFR China (Platts) Average Price Option</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>A38</t>
+          <t>ICT</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -1638,12 +1638,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Copper London TAM</t>
+          <t>London Spot Silver Futures</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>HGF</t>
+          <t>SSP</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -1655,12 +1655,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Gold Option</t>
+          <t>Copper TAS Futures</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>OG</t>
+          <t>HGT</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -1672,12 +1672,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Silver Option</t>
+          <t>Aluminium European Premium Duty-Unpaid (Metal Bulletin) Futures</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -1689,12 +1689,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Platinum Option</t>
+          <t>Copper Premium Grade A CIF Shanghai (Metal Bulletin) Futures</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PO</t>
+          <t>CUP</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1706,12 +1706,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Copper Spot TAS Futures</t>
+          <t>Copper Financial Futures</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>HG0</t>
+          <t>HGS</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1723,12 +1723,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>U.S. Midwest Busheling Ferrous Scrap (AMM) Futures</t>
+          <t>Micro Platinum Futures</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>BUS</t>
+          <t>PLM</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1740,12 +1740,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Silver TAS Futures</t>
+          <t>Gold Kilo Futures</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SIT</t>
+          <t>GCK</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1757,12 +1757,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Boston Real Estate Futures</t>
+          <t>San Francisco Real Estate Futures</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>SFR</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -1791,12 +1791,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Las Vegas Real Estate Futures</t>
+          <t>San Diego Real Estate Futures</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>LAV</t>
+          <t>SDG</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -1808,12 +1808,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CME Metro Area Housing Index Futures</t>
+          <t>Las Vegas Real Estate Futures</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>CUS</t>
+          <t>LAV</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -1825,12 +1825,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>New York Real Estate Futures</t>
+          <t>Washington DC Real Estate Futures</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -1842,12 +1842,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Chicago Real Estate Futures</t>
+          <t>Miami Real Estate Futures</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>CHI</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -1859,12 +1859,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>San Diego Real Estate Futures</t>
+          <t>CME Metro Area Housing Index Futures</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SDG</t>
+          <t>CUS</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -1876,12 +1876,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Los Angeles Real Estate Futures</t>
+          <t>New York Real Estate Futures</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>NYM</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -1893,12 +1893,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>San Francisco Real Estate Futures</t>
+          <t>Boston Real Estate Futures</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SFR</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -1910,12 +1910,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Washington DC Real Estate Futures</t>
+          <t>Los Angeles Real Estate Futures</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -1927,12 +1927,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Miami Real Estate Futures</t>
+          <t>Chicago Real Estate Futures</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>CHI</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -1944,12 +1944,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Portland HDD Q4 Seasonal Strip Options</t>
+          <t>Cincinnati CDD JUL Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>4H7</t>
+          <t>K3N</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -1961,12 +1961,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Tokyo CAT DEC Seasonal Strip Options</t>
+          <t>Essen CAT Q3 Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>G6Z</t>
+          <t>3G4</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -1978,12 +1978,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Las Vegas CDD Monthly Futures</t>
+          <t>New York HDD Q4 Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>K0</t>
+          <t>4H4</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -1995,12 +1995,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Minneapolis HDD NOV Seasonal Strip Options</t>
+          <t>Houston CDD Jul Seasonal Strip Futures</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>HQX</t>
+          <t>KRN</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2012,12 +2012,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Amsterdam CAT Monthly Options</t>
+          <t>Minneapolis HDD Q1 Seasonal Strip Futures</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>1HQ</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2029,12 +2029,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>New York HDD Q4 Seasonal Strip Futures</t>
+          <t>Portland HDD NOV Seasonal Strip Futures</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>4H4</t>
+          <t>H7X</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2046,12 +2046,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Tokyo CAT Q2 Seasonal Strip Options</t>
+          <t>Amsterdam HDD NOV Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>G62</t>
+          <t>D2X</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2063,12 +2063,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Atlanta HDD Q1 Seasonal Strip Options</t>
+          <t>Amsterdam HDD Q4 Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>1H1</t>
+          <t>4D2</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2080,12 +2080,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Cincinnati CDD MAY Seasonal Strip Options</t>
+          <t>Philadelphia CDD Index Futures</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>K3K</t>
+          <t>K6</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2097,12 +2097,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Atlanta HDD Q1 Seasonal Strip Futures</t>
+          <t>Paris CAT Jul Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>1H1</t>
+          <t>G1N</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2114,12 +2114,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>London HDD NOV Seasonal Strip Options</t>
+          <t>Sacramento HDD Monthly Options</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>D0X</t>
+          <t>HS</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">

</xml_diff>

<commit_message>
Final Backend Codes for Feature1
</commit_message>
<xml_diff>
--- a/backend/Data/finaldata.xlsx
+++ b/backend/Data/finaldata.xlsx
@@ -448,12 +448,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BTIC on S&amp;P-GSCI Commodity Index Futures</t>
+          <t>Soybean Meal TAS Futures</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GDT</t>
+          <t>ZMT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -465,12 +465,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cash-Settled Cheese Futures</t>
+          <t>Live Cattle Futures</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CSC</t>
+          <t>LE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -482,12 +482,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Chicago SRW Wheat-Corn ICS Synthetic Futures</t>
+          <t>KC HRW Wheat Futures</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>QCW</t>
+          <t>KE</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -499,12 +499,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Urea US Gulf Options</t>
+          <t>Corn Mar-Jul CSO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UGO</t>
+          <t>CZ7</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -516,12 +516,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DAP FOB NOLA Futures</t>
+          <t>Chicago SRW Wheat-Corn ICS Synthetic Futures</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DFN</t>
+          <t>QCW</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -533,12 +533,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Soybean Nov-July CSO</t>
+          <t>Corn July-Dec CSO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SZ9</t>
+          <t>CZ6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -550,12 +550,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Oats Options</t>
+          <t>MAP CFR Brazil Futures</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>OZO</t>
+          <t>MFC</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -567,12 +567,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MGEX-Chicago SRW Wheat Spread Synthetic Futures</t>
+          <t>Class III Milk Options</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MCX</t>
+          <t>DC</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -584,12 +584,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Soybean Oil Futures</t>
+          <t>MGEX-Chicago SRW Wheat Spread Synthetic Futures</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ZL</t>
+          <t>MCX</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -601,12 +601,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Consecutive Chicago SRW Wheat CSO</t>
+          <t>Short-Dated New Crop Soybean Options</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CZW</t>
+          <t>OSD</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -618,12 +618,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Short-Dated New Crop Soybean Meal Options</t>
+          <t>Soybean Oil Aug-Dec CSO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>OMD</t>
+          <t>NC4</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -635,12 +635,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Monthly Options on Micro Ether Futures</t>
+          <t>Ether/Bitcoin Ratio Futures</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>VM</t>
+          <t>EBR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -652,12 +652,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BTIC on Bitcoin Friday Futures</t>
+          <t>Ether Futures</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BFB</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -669,12 +669,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BTIC on Bitcoin futures against APAC Close (Bitcoin Reference Rate APAC - BRRAP)</t>
+          <t>Micro Bitcoin Euro Futures</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ABB</t>
+          <t>EBM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -686,12 +686,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TAS on Bitcoin Futures</t>
+          <t>BTIC on Ether Futures New York Close</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TBT</t>
+          <t>ENB</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -703,12 +703,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Monthly Options on Micro Bitcoin Futures</t>
+          <t>Micro Ether Futures</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>WM</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -720,12 +720,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BTIC on Micro Bitcoin Futures New York Close</t>
+          <t>Bitcoin Euro Futures</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MYB</t>
+          <t>BTE</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -737,12 +737,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bitcoin Friday Futures</t>
+          <t>Ether Euro Futures</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BFF</t>
+          <t>ETE</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -754,12 +754,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BTIC on Micro Ether Futures New York Close</t>
+          <t>BTIC on Bitcoin Futures London Close</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>EYB</t>
+          <t>BTB</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -771,12 +771,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Micro Bitcoin Euro Futures</t>
+          <t>BTIC on Bitcoin Friday Futures</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>EBM</t>
+          <t>BFB</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -805,12 +805,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Micro Ether Euro Futures</t>
+          <t>BTIC on Micro Ether futures against APAC Close (Ether-Dollar Reference Rate APAC - ETHUSD_AP)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EEM</t>
+          <t>AHB</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -822,12 +822,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Bakken Cushing (Argus) vs. WTI Trade Month Futures</t>
+          <t>Mont Belvieu LDH Propane (OPIS) vs. Argus Propane Far East Index Futures</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BKT</t>
+          <t>PMF</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -839,12 +839,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Gasoil 0.1% Cargoes CIF NWE (Platts) vs. Low Sulphur Gasoil BALMO Futures</t>
+          <t>Singapore Jet Kerosene (Platts) vs. Gasoil (Platts) BALMO Futures</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4V</t>
+          <t>AZ0</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -856,12 +856,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mini Japan C&amp;F Naphtha (Platts) Futures</t>
+          <t>Mini ULSD 10ppm Cargoes CIF MED (Platts) vs. Low Sulphur Gasoil Futures</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MJN</t>
+          <t>UCM</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -873,12 +873,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PJM METED Zone Off-Peak Calendar-Month Day-Ahead LMP Futures</t>
+          <t>PJM AECO Zone Peak Calendar-Day 5 MW Day-Ahead LMP Futures</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>A46</t>
+          <t>JPP</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -890,12 +890,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Japan C&amp;F Naphtha (Platts) Futures</t>
+          <t>Natural Gas Short-Term Option D15</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>JA</t>
+          <t>U15</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -907,12 +907,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>NY Harbor ULSD BALMO Futures</t>
+          <t>MISO Indiana Hub (formerly Cinergy Hub) Real-Time Off-Peak Calendar-Month 5 MW Futures</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>A1G</t>
+          <t>EJL</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -924,12 +924,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Los Angeles CARB Diesel (OPIS) Futures</t>
+          <t>ERCOT South 345 kV Hub 5 MW Off-Peak Calendar-Day Futures</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ALX</t>
+          <t>AM1</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -941,12 +941,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Mini Gasoil 0.1% Cargoes CIF NWE (Platts) vs. Low Sulphur Gasoil Futures</t>
+          <t>Jet Aviation Fuel Cargoes FOB MED (Platts) Futures</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MGF</t>
+          <t>1T</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -958,12 +958,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Micro Crude Oil TAS</t>
+          <t>RBOB Gasoline Bullet Futures</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MCT</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -975,12 +975,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ERCOT North 345 kV Hub 5 MW Peak Futures</t>
+          <t>Singapore Gasoil (Platts) BALMO Futures</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AI5</t>
+          <t>AVU</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -992,12 +992,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Singapore Gasoline 92 Unleaded (Platts) vs Gasoline Eurobob Non-Oxy NWE Barges (Argus) Futures</t>
+          <t>Middle East Gasoil FOB Arab Gulf (Platts) BALMO Futures</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SGF</t>
+          <t>MBS</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1009,12 +1009,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BTIC FTSE 100 Index (GBP) Futures</t>
+          <t>BTIC on E-mini Health Care Select Sector Futures</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>FTT</t>
+          <t>XVT</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1026,12 +1026,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>E-mini FTSE Emerging Index Futures</t>
+          <t>E-mini Dow Jones Industrial Average Options</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>EI</t>
+          <t>OYM</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1043,12 +1043,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>BTIC on E-mini S&amp;P Oil &amp; Gas Exploration &amp; Production Select Industry Futures</t>
+          <t>Micro E-mini Dow Jones Industrial Average Index Futures</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SWT</t>
+          <t>MYM</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1060,12 +1060,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>E-mini Industrial Select Sector Futures</t>
+          <t>TACO+ Futures on E-mini S&amp;P 500 Stock Price Index Futures</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>XAI</t>
+          <t>EQ1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1077,12 +1077,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>E-mini S&amp;P 500 Equal Weight Futures</t>
+          <t>BTIC on E-mini S&amp;P Oil &amp; Gas Exploration &amp; Production Select Industry Futures</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>EWF</t>
+          <t>SWT</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1094,12 +1094,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>BTIC on S&amp;P 500 Total Return Index Futures</t>
+          <t>E-mini Nikkei 225 (JPY) Futures</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TRB</t>
+          <t>ENY</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1111,12 +1111,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>S&amp;P 500 Growth Futures</t>
+          <t>BTIC on E-mini Russell 1000 Growth Futures</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>RGT</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1128,12 +1128,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Dow Jones Real Estate BTIC Futures</t>
+          <t>E-mini S&amp;P 500 EOM Options</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>REX</t>
+          <t>EW</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1145,12 +1145,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BTIC on E-mini Consumer Staples Select Sector Futures</t>
+          <t>Dow Jones Real Estate BTIC Futures</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>XPT</t>
+          <t>REX</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1162,12 +1162,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>BTIC E-mini S&amp;P 500 Futures</t>
+          <t>Dow Jones U.S. Real Estate Index Options</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>EST</t>
+          <t>RX</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1179,12 +1179,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>E-mini Russell 2000 Index Futures</t>
+          <t>E-mini Russell 1000 Growth Index Futures</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>RSG</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1196,12 +1196,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Australian Dollar Futures</t>
+          <t>Czech Koruna Futures</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>6A</t>
+          <t>CZK</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1213,12 +1213,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Russian Ruble Futures</t>
+          <t>Australian Dollar Futures</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>6R</t>
+          <t>6A</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1230,12 +1230,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Czech Koruna/Euro (CZK/EUR) Cross Rate Futures</t>
+          <t>E-mini Euro FX Futures</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ECK</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1247,12 +1247,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Chinese Renminbi/Euro Futures</t>
+          <t>Micro EUR/USD Futures</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>RME</t>
+          <t>M6E</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1264,12 +1264,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Turkish Lira/US Dollar (TRY/USD) Future</t>
+          <t>Euro/Swiss Franc Futures</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TRL</t>
+          <t>RF</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1281,12 +1281,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>USD/CNH Monthly Options</t>
+          <t>PLN/USD Monthly Options</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CNH</t>
+          <t>PLZ</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1298,12 +1298,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Australian Dollar/Japanese Yen Futures</t>
+          <t>Japanese Yen Futures</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>AJY</t>
+          <t>6J</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1315,12 +1315,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Micro AUD/USD Futures</t>
+          <t>KRW/USD Monthly Options</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>M6A</t>
+          <t>KRW</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1332,12 +1332,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>New Zealand Dollar Futures</t>
+          <t>Russian Ruble Futures</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>6N</t>
+          <t>6R</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1349,12 +1349,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Brazilian Real Futures</t>
+          <t>Polish Zloty Futures</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>6L</t>
+          <t>PLN</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1366,12 +1366,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Euro/Japanese Yen Futures</t>
+          <t>New Zealand Dollar Futures</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>RY</t>
+          <t>6N</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1383,12 +1383,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>5-Year MAC SOFR Swap Futures</t>
+          <t>30-Year UMBS TBA Futures - 2.0% Coupon</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>F1S</t>
+          <t>20U</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1400,12 +1400,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>5-Year Yield Futures</t>
+          <t>One-Year Mid-Curve Options on Three-Month SOFR Futures</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>5YY</t>
+          <t>S0</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1417,12 +1417,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>20-Year MAC SOFR Swap Futures</t>
+          <t>10-Year T-Note Options</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>E1S</t>
+          <t>OZN</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1434,12 +1434,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>30-Year UMBS TBA Futures - 4.5% Coupon</t>
+          <t>30-Year UMBS TBA Futures - 3.0% Coupon</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>45U</t>
+          <t>30U</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1451,12 +1451,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2-Year Yield Futures</t>
+          <t>30-Year UMBS TBA Futures - 4.5% Coupon</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2YY</t>
+          <t>45U</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1468,12 +1468,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>30-Year UMBS TBA Futures - 2.0% Coupon</t>
+          <t>Euro Short-Term Rate (€STR) - Three-Month Single Contract Basis Spread Futures</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>20U</t>
+          <t>EUS</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1485,12 +1485,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2-Year T-Note Options</t>
+          <t>ESTR Futures</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>OZT</t>
+          <t>ESR</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1502,12 +1502,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Ultra U.S. Treasury Bond Futures</t>
+          <t>Three-Month SOFR Futures</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>UB</t>
+          <t>SR3</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1519,12 +1519,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ESTR Futures</t>
+          <t>Four-Year Mid-Curve Options on Three-Month SOFR Futures</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ESR</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1536,12 +1536,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2-Year MAC SOFR Swap Futures</t>
+          <t>30-Year Eris SOFR Swap Futures</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>T1S</t>
+          <t>YIE</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1553,12 +1553,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>TAS on 2-Year Treasury Note Futures</t>
+          <t>4-Year Eris SOFR Swap Futures</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ZTT</t>
+          <t>YID</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1570,12 +1570,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Micro Gold TAS Futures</t>
+          <t>Iron Ore 62% Fe, CFR China (Platts) Average Price Option</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MGT</t>
+          <t>ICT</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1587,12 +1587,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Shanghai Gold (USD) Futures</t>
+          <t>Copper Premium Grade A CIF Shanghai (Metal Bulletin) Futures</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>SGU</t>
+          <t>CUP</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1604,12 +1604,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Spodumene CIF China (Fastmarkets) Futures</t>
+          <t>Aluminium European Premium Duty-Unpaid (Metal Bulletin) Futures</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>SPM</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1621,12 +1621,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Iron Ore 62% Fe, CFR China (Platts) Average Price Option</t>
+          <t>Gold London Trade At Marker First PM</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ICT</t>
+          <t>GCD</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -1638,12 +1638,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>London Spot Silver Futures</t>
+          <t>Copper Average Price Option</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>SSP</t>
+          <t>CAP</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -1655,12 +1655,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Copper TAS Futures</t>
+          <t>U.S. Midwest Domestic Hot-Rolled Coil Steel (CRU) Index Average Price Option</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>HGT</t>
+          <t>HRO</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -1672,12 +1672,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Aluminium European Premium Duty-Unpaid (Metal Bulletin) Futures</t>
+          <t>U.S. Midwest Domestic Steel Premium (CRU) Futures</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>HDG</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -1689,12 +1689,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Copper Premium Grade A CIF Shanghai (Metal Bulletin) Futures</t>
+          <t>Copper Futures</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>CUP</t>
+          <t>HG</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1706,12 +1706,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Copper Financial Futures</t>
+          <t>Alumina FOB Australia (Metal Bulletin) Futures</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>HGS</t>
+          <t>ALB</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1723,12 +1723,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Micro Platinum Futures</t>
+          <t>London Spot Silver Futures</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PLM</t>
+          <t>SSP</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1740,12 +1740,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Gold Kilo Futures</t>
+          <t>London Spot Gold Futures</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>GCK</t>
+          <t>GSP</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1757,12 +1757,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>San Francisco Real Estate Futures</t>
+          <t>CME Metro Area Housing Index Futures</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SFR</t>
+          <t>CUS</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -1774,12 +1774,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Denver Real Estate Futures</t>
+          <t>Miami Real Estate Futures</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -1791,12 +1791,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>San Diego Real Estate Futures</t>
+          <t>Los Angeles Real Estate Futures</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SDG</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -1808,12 +1808,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Las Vegas Real Estate Futures</t>
+          <t>New York Real Estate Futures</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>LAV</t>
+          <t>NYM</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -1825,12 +1825,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Washington DC Real Estate Futures</t>
+          <t>Boston Real Estate Futures</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -1842,12 +1842,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Miami Real Estate Futures</t>
+          <t>Las Vegas Real Estate Futures</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>LAV</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -1859,12 +1859,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CME Metro Area Housing Index Futures</t>
+          <t>San Diego Real Estate Futures</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>CUS</t>
+          <t>SDG</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -1876,12 +1876,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>New York Real Estate Futures</t>
+          <t>Washington DC Real Estate Futures</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -1893,12 +1893,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Boston Real Estate Futures</t>
+          <t>Chicago Real Estate Futures</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>CHI</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -1910,12 +1910,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Los Angeles Real Estate Futures</t>
+          <t>Denver Real Estate Futures</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -1927,12 +1927,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Chicago Real Estate Futures</t>
+          <t>San Francisco Real Estate Futures</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>CHI</t>
+          <t>SFR</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -1944,12 +1944,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Cincinnati CDD JUL Seasonal Strip Options</t>
+          <t>Essen CAT Q3 Seasonal Strip Futures</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>K3N</t>
+          <t>3G4</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -1961,12 +1961,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Essen CAT Q3 Seasonal Strip Options</t>
+          <t>Philadelphia HDD Dec Seasonal Strip Futures</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>3G4</t>
+          <t>H6Z</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -1978,12 +1978,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>New York HDD Q4 Seasonal Strip Options</t>
+          <t>Houston HDD Q4 Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>4H4</t>
+          <t>4HR</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -1995,12 +1995,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Houston CDD Jul Seasonal Strip Futures</t>
+          <t>Amsterdam HDD NOV Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>KRN</t>
+          <t>D2X</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2012,12 +2012,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Minneapolis HDD Q1 Seasonal Strip Futures</t>
+          <t>London HDD Q1 Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>1HQ</t>
+          <t>1D0</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2029,12 +2029,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Portland HDD NOV Seasonal Strip Futures</t>
+          <t>Philadelphia CDD Index Options</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>H7X</t>
+          <t>K6</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2046,12 +2046,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Amsterdam HDD NOV Seasonal Strip Options</t>
+          <t>Essen CAT Index Futures</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>D2X</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2063,12 +2063,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Amsterdam HDD Q4 Seasonal Strip Options</t>
+          <t>Sacramento HDD Q1 Seasonal Strip Futures</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>4D2</t>
+          <t>1HS</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2080,12 +2080,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Philadelphia CDD Index Futures</t>
+          <t>Tokyo CAT Q1 Seasonal Strip Futures</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>K6</t>
+          <t>1G6</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2097,12 +2097,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Paris CAT Jul Seasonal Strip Options</t>
+          <t>New York CDD JUL Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>G1N</t>
+          <t>K4N</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2114,12 +2114,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Sacramento HDD Monthly Options</t>
+          <t>Dallas CDD MAY Seasonal Strip Futures</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>HS</t>
+          <t>K5K</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">

</xml_diff>

<commit_message>
Final Updated Code for first Feature
</commit_message>
<xml_diff>
--- a/backend/Data/finaldata.xlsx
+++ b/backend/Data/finaldata.xlsx
@@ -448,12 +448,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Soybean Meal TAS Futures</t>
+          <t>Black Sea Corn Financially Settled (Platts) Options</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ZMT</t>
+          <t>BSO</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -465,12 +465,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Live Cattle Futures</t>
+          <t>Chicago SRW Wheat Dec-July CSO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LE</t>
+          <t>WC6</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -482,12 +482,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>KC HRW Wheat Futures</t>
+          <t>Chicago SRW Wheat-Corn ICS Synthetic Futures</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>KE</t>
+          <t>QCW</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -499,12 +499,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Corn Mar-Jul CSO</t>
+          <t>Class III Milk Options</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CZ7</t>
+          <t>DC</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -516,12 +516,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Chicago SRW Wheat-Corn ICS Synthetic Futures</t>
+          <t>Corn Mar-Dec CSO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>QCW</t>
+          <t>CZ9</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -533,12 +533,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Corn July-Dec CSO</t>
+          <t>Mini Soybean Futures</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CZ6</t>
+          <t>XK</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -550,12 +550,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MAP CFR Brazil Futures</t>
+          <t>Corn July-Dec CSO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MFC</t>
+          <t>CZ6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -567,12 +567,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Class III Milk Options</t>
+          <t>Lean Hog Futures</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DC</t>
+          <t>HE</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -584,12 +584,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MGEX-Chicago SRW Wheat Spread Synthetic Futures</t>
+          <t>Feeder Cattle Options</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MCX</t>
+          <t>GF</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -601,12 +601,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Short-Dated New Crop Soybean Options</t>
+          <t>Short-Dated New Crop KC HRW Wheat Options</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>OSD</t>
+          <t>KWE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -618,12 +618,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Soybean Oil Aug-Dec CSO</t>
+          <t>Corn Futures</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NC4</t>
+          <t>ZC</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -635,12 +635,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ether/Bitcoin Ratio Futures</t>
+          <t>Micro Ether Euro Futures</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>EBR</t>
+          <t>EEM</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -652,12 +652,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ether Futures</t>
+          <t>TAS on Bitcoin Futures</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>TBT</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -669,12 +669,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Micro Bitcoin Euro Futures</t>
+          <t>BTIC on Micro Ether futures against APAC Close (Ether-Dollar Reference Rate APAC - ETHUSD_AP)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>EBM</t>
+          <t>AHB</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -686,12 +686,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BTIC on Ether Futures New York Close</t>
+          <t>Ether Futures</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ENB</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -703,12 +703,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Micro Ether Futures</t>
+          <t>BTIC on Bitcoin Futures London Close</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>BTB</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -720,12 +720,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Bitcoin Euro Futures</t>
+          <t>Options on Ether Futures</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>BTE</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -737,12 +737,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ether Euro Futures</t>
+          <t>Bitcoin Friday Futures</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ETE</t>
+          <t>BFF</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -754,12 +754,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BTIC on Bitcoin Futures London Close</t>
+          <t>BTIC on Ether Futures London Close</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BTB</t>
+          <t>ETB</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -771,12 +771,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BTIC on Bitcoin Friday Futures</t>
+          <t>TAS on Micro Bitcoin Futures</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BFB</t>
+          <t>TBM</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -788,12 +788,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BTIC on Micro Ether Futures London Close</t>
+          <t>BTIC on Bitcoin Friday Futures</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>EMB</t>
+          <t>BFB</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -805,12 +805,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BTIC on Micro Ether futures against APAC Close (Ether-Dollar Reference Rate APAC - ETHUSD_AP)</t>
+          <t>BTIC on Bitcoin futures against APAC Close (Bitcoin Reference Rate APAC - BRRAP)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>AHB</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -822,12 +822,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mont Belvieu LDH Propane (OPIS) vs. Argus Propane Far East Index Futures</t>
+          <t>WTI Houston (Argus) vs. Brent Trade Month Futures</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PMF</t>
+          <t>WHB</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -839,12 +839,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Singapore Jet Kerosene (Platts) vs. Gasoil (Platts) BALMO Futures</t>
+          <t>Crude Oil 5 Year MidCurve Option</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AZ0</t>
+          <t>LM5</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -856,12 +856,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mini ULSD 10ppm Cargoes CIF MED (Platts) vs. Low Sulphur Gasoil Futures</t>
+          <t>Guernsey Light Sweet (Argus) Monthly Futures</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>UCM</t>
+          <t>GSW</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -873,12 +873,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PJM AECO Zone Peak Calendar-Day 5 MW Day-Ahead LMP Futures</t>
+          <t>Natural Gas (Henry Hub) Last-day Financial 2 Month Spread Option</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>JPP</t>
+          <t>AG2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -890,12 +890,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Natural Gas Short-Term Option D15</t>
+          <t>Daily Natural Gas Option</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>U15</t>
+          <t>KDB</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -907,12 +907,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MISO Indiana Hub (formerly Cinergy Hub) Real-Time Off-Peak Calendar-Month 5 MW Futures</t>
+          <t>Container Freight (China/East Asia to US West Coast) (FBX01) (Baltic) Futures</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EJL</t>
+          <t>CS1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -924,12 +924,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ERCOT South 345 kV Hub 5 MW Off-Peak Calendar-Day Futures</t>
+          <t>Japanese Power (Day-Ahead) Tokyo Peak-Load Futures</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>AM1</t>
+          <t>JPT</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -941,12 +941,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Jet Aviation Fuel Cargoes FOB MED (Platts) Futures</t>
+          <t>Mini European Jet Kero Barges FOB Rdam (Platts) vs. Low Sulphur Gasoil Futures</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1T</t>
+          <t>MJB</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -958,12 +958,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>RBOB Gasoline Bullet Futures</t>
+          <t>NYISO Zone J Day-Ahead Peak Calendar-Month 5 MW Option</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>9AV</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -975,12 +975,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Singapore Gasoil (Platts) BALMO Futures</t>
+          <t>Group Three ULSD (Platts) vs. NY Harbor ULSD Futures</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AVU</t>
+          <t>AA6</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -992,12 +992,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Middle East Gasoil FOB Arab Gulf (Platts) BALMO Futures</t>
+          <t>CBL California Carbon Allowance Vintage-Specific Futures 2023</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>MBS</t>
+          <t>CC3</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1009,12 +1009,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BTIC on E-mini Health Care Select Sector Futures</t>
+          <t>BTIC on Adjusted Interest Rate S&amp;P 500 Total Return (SOFR) Futures</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>XVT</t>
+          <t>ASPT</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1026,12 +1026,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>E-mini Dow Jones Industrial Average Options</t>
+          <t>E-mini Utilities Select Sector Futures</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>OYM</t>
+          <t>XAU</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1043,12 +1043,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Micro E-mini Dow Jones Industrial Average Index Futures</t>
+          <t>BTIC on E-mini S&amp;P Oil &amp; Gas Exploration &amp; Production Select Industry Futures</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MYM</t>
+          <t>SWT</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1060,12 +1060,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TACO+ Futures on E-mini S&amp;P 500 Stock Price Index Futures</t>
+          <t>E-mini S&amp;P 500 EOM Options</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EQ1</t>
+          <t>EW</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1077,12 +1077,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>BTIC on E-mini S&amp;P Oil &amp; Gas Exploration &amp; Production Select Industry Futures</t>
+          <t>E-mini S&amp;P 500 Futures</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SWT</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1094,12 +1094,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>E-mini Nikkei 225 (JPY) Futures</t>
+          <t>E-mini Communication Services Select Sector Futures</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ENY</t>
+          <t>XAZ</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1111,12 +1111,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>BTIC on E-mini Russell 1000 Growth Futures</t>
+          <t>E-mini Nikkei 225 (JPY) Futures</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>RGT</t>
+          <t>ENY</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1128,12 +1128,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>E-mini S&amp;P 500 EOM Options</t>
+          <t>Micro E-mini S&amp;P 500 Options</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>EW</t>
+          <t>MES</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1145,12 +1145,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Dow Jones Real Estate BTIC Futures</t>
+          <t>Nasdaq Veles California Water Index Futures</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>REX</t>
+          <t>H2O</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1162,12 +1162,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Dow Jones U.S. Real Estate Index Options</t>
+          <t>Nikkei (USD) Futures</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>RX</t>
+          <t>NKD</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1179,12 +1179,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>E-mini Russell 1000 Growth Index Futures</t>
+          <t>BTIC on E-mini Financial Select Sector Futures</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>RSG</t>
+          <t>XFT</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1196,12 +1196,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Czech Koruna Futures</t>
+          <t>Japanese Yen Futures</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CZK</t>
+          <t>6J</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1213,12 +1213,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Australian Dollar Futures</t>
+          <t>Euro/Norwegian Krone Futures</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>6A</t>
+          <t>ENK</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1230,12 +1230,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>E-mini Euro FX Futures</t>
+          <t>Mexican Peso Futures</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>6M</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1247,12 +1247,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Micro EUR/USD Futures</t>
+          <t>Chinese Renminbi/USD Futures</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>M6E</t>
+          <t>RMB</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1264,12 +1264,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Euro/Swiss Franc Futures</t>
+          <t>Russian Ruble Futures</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>RF</t>
+          <t>6R</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1281,12 +1281,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PLN/USD Monthly Options</t>
+          <t>RUB/USD Monthly Options</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PLZ</t>
+          <t>6R</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1298,12 +1298,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Japanese Yen Futures</t>
+          <t>Norwegian Krone Futures</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>6J</t>
+          <t>NOK</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1315,12 +1315,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>KRW/USD Monthly Options</t>
+          <t>JPY/USD Monthly Options</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>KRW</t>
+          <t>JPU</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1332,12 +1332,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Russian Ruble Futures</t>
+          <t>GBP/CAD Futures</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>6R</t>
+          <t>PCD</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1349,12 +1349,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Polish Zloty Futures</t>
+          <t>Korean Won Futures</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PLN</t>
+          <t>KRW</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1366,12 +1366,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>New Zealand Dollar Futures</t>
+          <t>Micro EUR/USD Futures</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>6N</t>
+          <t>M6E</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1383,12 +1383,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>30-Year UMBS TBA Futures - 2.0% Coupon</t>
+          <t>30-Year UMBS TBA Futures - 2.5% Coupon</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>20U</t>
+          <t>25U</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1400,12 +1400,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>One-Year Mid-Curve Options on Three-Month SOFR Futures</t>
+          <t>BTIC on Bloomberg IG Credit Futures</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>S0</t>
+          <t>IQBT</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1417,12 +1417,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>10-Year T-Note Options</t>
+          <t>Three-Year Mid-Curve Options on Three-Month SOFR Futures</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>OZN</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1434,12 +1434,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>30-Year UMBS TBA Futures - 3.0% Coupon</t>
+          <t>Ultra U.S. Treasury Bond Options</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>30U</t>
+          <t>OUB</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1451,12 +1451,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>30-Year UMBS TBA Futures - 4.5% Coupon</t>
+          <t>30-Year UMBS TBA Futures - 6.5% Coupon</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>45U</t>
+          <t>65U</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1468,12 +1468,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Euro Short-Term Rate (€STR) - Three-Month Single Contract Basis Spread Futures</t>
+          <t>10-Year T-Note Futures</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>EUS</t>
+          <t>ZN</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1485,12 +1485,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ESTR Futures</t>
+          <t>Four-Year Mid-Curve Options on Three-Month SOFR Futures</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ESR</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1502,12 +1502,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Three-Month SOFR Futures</t>
+          <t>30-Year MAC SOFR Swap Futures</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SR3</t>
+          <t>B1S</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1519,12 +1519,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Four-Year Mid-Curve Options on Three-Month SOFR Futures</t>
+          <t>Two-Year Mid-Curve Options on Three-Month SOFR Futures</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1536,12 +1536,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>30-Year Eris SOFR Swap Futures</t>
+          <t>2-Year Eris SOFR Swap Futures</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>YIE</t>
+          <t>YIT</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1553,12 +1553,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>4-Year Eris SOFR Swap Futures</t>
+          <t>30-Year UMBS TBA Futures - 5.5% Coupon</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>YID</t>
+          <t>55U</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1570,12 +1570,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Iron Ore 62% Fe, CFR China (Platts) Average Price Option</t>
+          <t>Aluminum Futures</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ICT</t>
+          <t>ALI</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1587,12 +1587,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Copper Premium Grade A CIF Shanghai (Metal Bulletin) Futures</t>
+          <t>Gold London Trade At Marker First PM</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>CUP</t>
+          <t>GCD</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1604,12 +1604,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Aluminium European Premium Duty-Unpaid (Metal Bulletin) Futures</t>
+          <t>Aluminum Option</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>AX</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1621,12 +1621,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Gold London Trade At Marker First PM</t>
+          <t>Aluminum MW U.S. Transaction Premium Platts (25MT) Average Price Option</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>GCD</t>
+          <t>ALO</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -1638,12 +1638,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Copper Average Price Option</t>
+          <t>Cobalt Metal (Fastmarkets) Average Price Option</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>CAP</t>
+          <t>COO</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -1655,12 +1655,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>U.S. Midwest Domestic Hot-Rolled Coil Steel (CRU) Index Average Price Option</t>
+          <t>Copper Option</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>HRO</t>
+          <t>HXE</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -1672,12 +1672,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>U.S. Midwest Domestic Steel Premium (CRU) Futures</t>
+          <t>E-mini Copper Futures</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>HDG</t>
+          <t>QC</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -1689,12 +1689,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Copper Futures</t>
+          <t>Lead Futures</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>HG</t>
+          <t>LED</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1706,12 +1706,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Alumina FOB Australia (Metal Bulletin) Futures</t>
+          <t>Lithium Hydroxide CIF CJK (Fastmarkets) Futures</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ALB</t>
+          <t>LTH</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1723,12 +1723,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>London Spot Silver Futures</t>
+          <t>London Spot Gold Futures</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SSP</t>
+          <t>GSP</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1740,12 +1740,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>London Spot Gold Futures</t>
+          <t>Iron Ore 62% Fe, CFR China (Platts) Futures</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>GSP</t>
+          <t>TIO</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1757,12 +1757,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CME Metro Area Housing Index Futures</t>
+          <t>Denver Real Estate Futures</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>CUS</t>
+          <t>DEN</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -1774,12 +1774,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Miami Real Estate Futures</t>
+          <t>San Francisco Real Estate Futures</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>SFR</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -1791,12 +1791,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Los Angeles Real Estate Futures</t>
+          <t>Chicago Real Estate Futures</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>LAX</t>
+          <t>CHI</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -1808,12 +1808,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>New York Real Estate Futures</t>
+          <t>CME Metro Area Housing Index Futures</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>CUS</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -1825,12 +1825,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Boston Real Estate Futures</t>
+          <t>Washington DC Real Estate Futures</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -1842,12 +1842,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Las Vegas Real Estate Futures</t>
+          <t>San Diego Real Estate Futures</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>LAV</t>
+          <t>SDG</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -1859,12 +1859,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>San Diego Real Estate Futures</t>
+          <t>Los Angeles Real Estate Futures</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SDG</t>
+          <t>LAX</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -1876,12 +1876,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Washington DC Real Estate Futures</t>
+          <t>Boston Real Estate Futures</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -1893,12 +1893,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Chicago Real Estate Futures</t>
+          <t>Las Vegas Real Estate Futures</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>CHI</t>
+          <t>LAV</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -1910,12 +1910,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Denver Real Estate Futures</t>
+          <t>Miami Real Estate Futures</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>DEN</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -1927,12 +1927,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>San Francisco Real Estate Futures</t>
+          <t>New York Real Estate Futures</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SFR</t>
+          <t>NYM</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -1944,12 +1944,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Essen CAT Q3 Seasonal Strip Futures</t>
+          <t>Atlanta HDD Q1 Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>3G4</t>
+          <t>1H1</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -1961,12 +1961,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Philadelphia HDD Dec Seasonal Strip Futures</t>
+          <t>Las Vegas CDD JUL Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>H6Z</t>
+          <t>K0N</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -1978,12 +1978,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Houston HDD Q4 Seasonal Strip Options</t>
+          <t>Essen CAT Index Futures</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>4HR</t>
+          <t>G4</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -1995,12 +1995,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Amsterdam HDD NOV Seasonal Strip Options</t>
+          <t>Paris CAT Q3 Seasonal Strip Futures</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>D2X</t>
+          <t>3G1</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2012,12 +2012,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>London HDD Q1 Seasonal Strip Options</t>
+          <t>Amsterdam HDD Q1 Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>1D0</t>
+          <t>1D2</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2029,12 +2029,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Philadelphia CDD Index Options</t>
+          <t>Las Vegas HDD Q4 Seasonal Strip Futures</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>K6</t>
+          <t>4H0</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2046,12 +2046,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Essen CAT Index Futures</t>
+          <t>London CAT Monthly Futures</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>G4</t>
+          <t>G0</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2063,12 +2063,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Sacramento HDD Q1 Seasonal Strip Futures</t>
+          <t>Minneapolis CDD Q2 Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>1HS</t>
+          <t>2KQ</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2080,12 +2080,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Tokyo CAT Q1 Seasonal Strip Futures</t>
+          <t>Atlanta CDD JUL Seasonal Strip Futures</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>1G6</t>
+          <t>K1N</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2097,12 +2097,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>New York CDD JUL Seasonal Strip Options</t>
+          <t>Portland HDD DEC Seasonal Strip Options</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>K4N</t>
+          <t>H7Z</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2114,12 +2114,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Dallas CDD MAY Seasonal Strip Futures</t>
+          <t>Dallas HDD DEC Seasonal Strip Futures</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>K5K</t>
+          <t>H5Z</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">

</xml_diff>